<commit_message>
feat(data): Group→Company→Facility hierarchy; company-level demand
- shipping: company = operator, group = Group Company (conglomerate, from
  clarkson) — facility (owner·engine) → company → group; demand at company level
  (owner total), so each operator optimises its own fleet under its own CO2 target
  while the group/all levels remain available for cap/demand scoping.
- steel: company = owner (POSCO / Hyundai Steel) → facility (plant); company-level
  steel demand (owner may allocate across its plants while transitioning).
- regenerated shipping.xlsx (per-company + ammonia/hydrogen) + steel.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/pathwise/public/examples/shipping.xlsx
+++ b/frontend/pathwise/public/examples/shipping.xlsx
@@ -10844,7 +10844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10860,10 +10860,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>baseline_technology</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>capacity</t>
         </is>
@@ -10882,10 +10887,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Dong-A Tanker Co</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -10902,10 +10912,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Dong-A Tanker Co</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -10922,10 +10937,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>86</v>
       </c>
     </row>
@@ -10942,10 +10962,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>IFO 380, Methanol</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10962,10 +10987,15 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>LPG, VLS IFO</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10982,10 +11012,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>22</v>
       </c>
     </row>
@@ -11002,10 +11037,15 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Hyundai Motor Group</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Biofuel</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11022,10 +11062,15 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Hyundai Motor Group</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>37</v>
       </c>
     </row>
@@ -11042,10 +11087,15 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Hyundai Motor Group</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -11062,10 +11112,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>KMTC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11082,10 +11137,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>KMTC</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11102,10 +11162,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Namsung Shipping</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>9</v>
       </c>
     </row>
@@ -11122,10 +11187,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Namsung Shipping</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11142,10 +11212,15 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Biofuel</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11162,10 +11237,15 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>IFO 180</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11182,10 +11262,15 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>89</v>
       </c>
     </row>
@@ -11202,10 +11287,15 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>LNG, VLS IFO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>19</v>
       </c>
     </row>
@@ -11222,10 +11312,15 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>LNG, VLS MGO</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11242,10 +11337,15 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>LPG, VLS IFO</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11262,10 +11362,15 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>261</v>
       </c>
     </row>
@@ -11282,10 +11387,15 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>VLS MDO</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11302,10 +11412,15 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Pan Ocean</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>IFO 180</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11322,10 +11437,15 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>Pan Ocean</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>38</v>
       </c>
     </row>
@@ -11342,10 +11462,15 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>Pan Ocean</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>51</v>
       </c>
     </row>
@@ -11362,10 +11487,15 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Hahn &amp; Company</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
         <v>38</v>
       </c>
     </row>
@@ -11382,10 +11512,15 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Hahn &amp; Company</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>LNG, VLS IFO</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>5</v>
       </c>
     </row>
@@ -11402,10 +11537,15 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>Hahn &amp; Company</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>3</v>
       </c>
     </row>
@@ -11422,10 +11562,15 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Sinokor Merchant</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>IFO 380</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
         <v>101</v>
       </c>
     </row>
@@ -11442,10 +11587,15 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>Sinokor Merchant</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>LNG, VLS IFO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11462,10 +11612,15 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>Sinokor Merchant</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>VLS IFO</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
         <v>68</v>
       </c>
     </row>

</xml_diff>